<commit_message>
Competencia Carmen: T1 piso 8 (Century 21, $200M, 57 m²)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018CaPYB92zD2dguENatYVXw
</commit_message>
<xml_diff>
--- a/finanzas/carmen_competencia_oct2026.xlsx
+++ b/finanzas/carmen_competencia_oct2026.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="53">
   <si>
     <t xml:space="preserve">Competencia — Carmen de Apicalá (conjunto Calle 1 # 11-10) · llamadas 9 oct 2026</t>
   </si>
@@ -152,7 +152,28 @@
     <t xml:space="preserve">Precio alterno dicho por abuelos: $250M amoblado</t>
   </si>
   <si>
-    <t xml:space="preserve">Metrocuadrado</t>
+    <t xml:space="preserve">Century 21 (ficha técnica, ID 149314)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beatriz Triviño · +57 302 702 3042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T1 / piso 8 (apto 805)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 privado cubierto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No dice (descripción no lo menciona)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inmobiliaria (Century 21)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excelente · construido 2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arenitas Riviera PH, Etapa 1. Balcón con vista. Precio de inmobiliaria: incluye su comisión.</t>
   </si>
   <si>
     <t xml:space="preserve">Letrero</t>
@@ -338,16 +359,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -355,55 +380,55 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -662,498 +687,522 @@
   <dimension ref="A1:V21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="30"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="K4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="L4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="M4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="N4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="O4" s="3" t="s">
+      <c r="O4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="P4" s="3" t="s">
+      <c r="P4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="Q4" s="3" t="s">
+      <c r="Q4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="R4" s="3" t="s">
+      <c r="R4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="S4" s="3" t="s">
+      <c r="S4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="T4" s="3" t="s">
+      <c r="T4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="U4" s="3" t="s">
+      <c r="U4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="V4" s="3" t="s">
+      <c r="V4" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4" t="s">
+      <c r="C5" s="5"/>
+      <c r="D5" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="6" t="n">
         <v>62.14</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="H5" s="7" t="n">
         <v>220000000</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="I5" s="7" t="n">
         <f aca="false">IFERROR(H5/E5,"")</f>
         <v>3540392.66173157</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="J5" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K5" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="L5" s="4" t="s">
+      <c r="L5" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M5" s="4" t="s">
+      <c r="M5" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="N5" s="4" t="s">
+      <c r="N5" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="O5" s="4" t="s">
+      <c r="O5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="P5" s="4" t="s">
+      <c r="P5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q5" s="4" t="s">
+      <c r="Q5" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="R5" s="6" t="s">
+      <c r="R5" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="S5" s="4" t="s">
+      <c r="S5" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="T5" s="6" t="s">
+      <c r="T5" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="U5" s="4" t="s">
+      <c r="U5" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="V5" s="4" t="s">
+      <c r="V5" s="5" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="12" t="str">
+      <c r="C6" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>57</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="12" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="I6" s="13" t="n">
         <f aca="false">IFERROR(H6/E6,"")</f>
-        <v/>
-      </c>
-      <c r="J6" s="13" t="str">
+        <v>3508771.92982456</v>
+      </c>
+      <c r="J6" s="14" t="n">
         <f aca="false">IFERROR(I6/$I$5-1,"")</f>
-        <v/>
-      </c>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="9"/>
-      <c r="Q6" s="9"/>
-      <c r="R6" s="11"/>
-      <c r="S6" s="9"/>
-      <c r="T6" s="11"/>
-      <c r="U6" s="9"/>
-      <c r="V6" s="9"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="n">
+        <v>-0.00893141945773524</v>
+      </c>
+      <c r="K6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="L6" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
+      <c r="O6" s="10"/>
+      <c r="P6" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q6" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="R6" s="12"/>
+      <c r="S6" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="T6" s="12"/>
+      <c r="U6" s="10"/>
+      <c r="V6" s="10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="12" t="str">
+      <c r="B7" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="13" t="str">
         <f aca="false">IFERROR(H7/E7,"")</f>
         <v/>
       </c>
-      <c r="J7" s="13" t="str">
+      <c r="J7" s="14" t="str">
         <f aca="false">IFERROR(I7/$I$5-1,"")</f>
         <v/>
       </c>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="9"/>
-      <c r="P7" s="9"/>
-      <c r="Q7" s="9"/>
-      <c r="R7" s="11"/>
-      <c r="S7" s="9"/>
-      <c r="T7" s="11"/>
-      <c r="U7" s="9"/>
-      <c r="V7" s="9"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="n">
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="10"/>
+      <c r="P7" s="10"/>
+      <c r="Q7" s="10"/>
+      <c r="R7" s="12"/>
+      <c r="S7" s="10"/>
+      <c r="T7" s="12"/>
+      <c r="U7" s="10"/>
+      <c r="V7" s="10"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="12" t="str">
+      <c r="B8" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="13" t="str">
         <f aca="false">IFERROR(H8/E8,"")</f>
         <v/>
       </c>
-      <c r="J8" s="13" t="str">
+      <c r="J8" s="14" t="str">
         <f aca="false">IFERROR(I8/$I$5-1,"")</f>
         <v/>
       </c>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="9"/>
-      <c r="Q8" s="9"/>
-      <c r="R8" s="11"/>
-      <c r="S8" s="9"/>
-      <c r="T8" s="11"/>
-      <c r="U8" s="9"/>
-      <c r="V8" s="9"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="n">
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
+      <c r="P8" s="10"/>
+      <c r="Q8" s="10"/>
+      <c r="R8" s="12"/>
+      <c r="S8" s="10"/>
+      <c r="T8" s="12"/>
+      <c r="U8" s="10"/>
+      <c r="V8" s="10"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="12" t="str">
+      <c r="B9" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="13" t="str">
         <f aca="false">IFERROR(H9/E9,"")</f>
         <v/>
       </c>
-      <c r="J9" s="13" t="str">
+      <c r="J9" s="14" t="str">
         <f aca="false">IFERROR(I9/$I$5-1,"")</f>
         <v/>
       </c>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="9"/>
-      <c r="Q9" s="9"/>
-      <c r="R9" s="11"/>
-      <c r="S9" s="9"/>
-      <c r="T9" s="11"/>
-      <c r="U9" s="9"/>
-      <c r="V9" s="9"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="n">
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10"/>
+      <c r="P9" s="10"/>
+      <c r="Q9" s="10"/>
+      <c r="R9" s="12"/>
+      <c r="S9" s="10"/>
+      <c r="T9" s="12"/>
+      <c r="U9" s="10"/>
+      <c r="V9" s="10"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="12" t="str">
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="13" t="str">
         <f aca="false">IFERROR(H10/E10,"")</f>
         <v/>
       </c>
-      <c r="J10" s="13" t="str">
+      <c r="J10" s="14" t="str">
         <f aca="false">IFERROR(I10/$I$5-1,"")</f>
         <v/>
       </c>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="9"/>
-      <c r="N10" s="9"/>
-      <c r="O10" s="9"/>
-      <c r="P10" s="9"/>
-      <c r="Q10" s="9"/>
-      <c r="R10" s="11"/>
-      <c r="S10" s="9"/>
-      <c r="T10" s="11"/>
-      <c r="U10" s="9"/>
-      <c r="V10" s="9"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="n">
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+      <c r="O10" s="10"/>
+      <c r="P10" s="10"/>
+      <c r="Q10" s="10"/>
+      <c r="R10" s="12"/>
+      <c r="S10" s="10"/>
+      <c r="T10" s="12"/>
+      <c r="U10" s="10"/>
+      <c r="V10" s="10"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="12" t="str">
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="13" t="str">
         <f aca="false">IFERROR(H11/E11,"")</f>
         <v/>
       </c>
-      <c r="J11" s="13" t="str">
+      <c r="J11" s="14" t="str">
         <f aca="false">IFERROR(I11/$I$5-1,"")</f>
         <v/>
       </c>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-      <c r="M11" s="9"/>
-      <c r="N11" s="9"/>
-      <c r="O11" s="9"/>
-      <c r="P11" s="9"/>
-      <c r="Q11" s="9"/>
-      <c r="R11" s="11"/>
-      <c r="S11" s="9"/>
-      <c r="T11" s="11"/>
-      <c r="U11" s="9"/>
-      <c r="V11" s="9"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="n">
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="10"/>
+      <c r="P11" s="10"/>
+      <c r="Q11" s="10"/>
+      <c r="R11" s="12"/>
+      <c r="S11" s="10"/>
+      <c r="T11" s="12"/>
+      <c r="U11" s="10"/>
+      <c r="V11" s="10"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="12" t="str">
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="13" t="str">
         <f aca="false">IFERROR(H12/E12,"")</f>
         <v/>
       </c>
-      <c r="J12" s="13" t="str">
+      <c r="J12" s="14" t="str">
         <f aca="false">IFERROR(I12/$I$5-1,"")</f>
         <v/>
       </c>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="9"/>
-      <c r="N12" s="9"/>
-      <c r="O12" s="9"/>
-      <c r="P12" s="9"/>
-      <c r="Q12" s="9"/>
-      <c r="R12" s="11"/>
-      <c r="S12" s="9"/>
-      <c r="T12" s="11"/>
-      <c r="U12" s="9"/>
-      <c r="V12" s="9"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="n">
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="10"/>
+      <c r="P12" s="10"/>
+      <c r="Q12" s="10"/>
+      <c r="R12" s="12"/>
+      <c r="S12" s="10"/>
+      <c r="T12" s="12"/>
+      <c r="U12" s="10"/>
+      <c r="V12" s="10"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="12" t="str">
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="13" t="str">
         <f aca="false">IFERROR(H13/E13,"")</f>
         <v/>
       </c>
-      <c r="J13" s="13" t="str">
+      <c r="J13" s="14" t="str">
         <f aca="false">IFERROR(I13/$I$5-1,"")</f>
         <v/>
       </c>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
-      <c r="M13" s="9"/>
-      <c r="N13" s="9"/>
-      <c r="O13" s="9"/>
-      <c r="P13" s="9"/>
-      <c r="Q13" s="9"/>
-      <c r="R13" s="11"/>
-      <c r="S13" s="9"/>
-      <c r="T13" s="11"/>
-      <c r="U13" s="9"/>
-      <c r="V13" s="9"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="14" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="B16" s="16" t="str">
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="10"/>
+      <c r="O13" s="10"/>
+      <c r="P13" s="10"/>
+      <c r="Q13" s="10"/>
+      <c r="R13" s="12"/>
+      <c r="S13" s="10"/>
+      <c r="T13" s="12"/>
+      <c r="U13" s="10"/>
+      <c r="V13" s="10"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="15" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="17" t="n">
         <f aca="false">IFERROR(AVERAGE(I6:I13),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="B17" s="16" t="n">
+        <v>3508771.92982456</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" s="17" t="n">
         <f aca="false">IFERROR(MIN(I6:I13),"")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="16" t="n">
+        <v>3508771.92982456</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="17" t="n">
         <f aca="false">IFERROR(MAX(I6:I13),"")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19" s="16" t="n">
+        <v>3508771.92982456</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="17" t="n">
         <f aca="false">I5</f>
         <v>3540392.66173157</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="B20" s="16" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="B20" s="17" t="n">
         <f aca="false">IFERROR(250000000/E5,"")</f>
         <v>4023173.47924043</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="B21" s="16" t="str">
+      <c r="C20" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" s="17" t="n">
         <f aca="false">IFERROR(B16*E5,"")</f>
-        <v/>
+        <v>218035087.719298</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Carmen: conjunto Arenitas Riviera PH, estrato 3; análisis de mercado oct en curso
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018CaPYB92zD2dguENatYVXw
</commit_message>
<xml_diff>
--- a/finanzas/carmen_competencia_oct2026.xlsx
+++ b/finanzas/carmen_competencia_oct2026.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="55">
   <si>
     <t xml:space="preserve">Competencia — Carmen de Apicalá (conjunto Calle 1 # 11-10) · llamadas 9 oct 2026</t>
   </si>
@@ -149,10 +149,13 @@
     <t xml:space="preserve">(pendiente)</t>
   </si>
   <si>
+    <t xml:space="preserve">3 (mismo conjunto: Arenitas Riviera PH)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Precio alterno dicho por abuelos: $250M amoblado</t>
   </si>
   <si>
-    <t xml:space="preserve">Century 21 (ficha técnica, ID 149314)</t>
+    <t xml:space="preserve">Letrero · Century 21 (ficha ID 149314)</t>
   </si>
   <si>
     <t xml:space="preserve">Beatriz Triviño · +57 302 702 3042</t>
@@ -174,6 +177,9 @@
   </si>
   <si>
     <t xml:space="preserve">Arenitas Riviera PH, Etapa 1. Balcón con vista. Precio de inmobiliaria: incluye su comisión.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metrocuadrado</t>
   </si>
   <si>
     <t xml:space="preserve">Letrero</t>
@@ -843,7 +849,7 @@
         <v>34</v>
       </c>
       <c r="S5" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="T5" s="7" t="s">
         <v>34</v>
@@ -852,7 +858,7 @@
         <v>29</v>
       </c>
       <c r="V5" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -860,13 +866,13 @@
         <v>1</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E6" s="11" t="n">
         <v>57</v>
@@ -889,19 +895,19 @@
         <v>-0.00893141945773524</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M6" s="10"/>
       <c r="N6" s="10"/>
       <c r="O6" s="10"/>
       <c r="P6" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q6" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="R6" s="12"/>
       <c r="S6" s="10" t="n">
@@ -910,7 +916,7 @@
       <c r="T6" s="12"/>
       <c r="U6" s="10"/>
       <c r="V6" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -918,7 +924,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
@@ -952,7 +958,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
@@ -986,7 +992,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
@@ -1145,12 +1151,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B16" s="17" t="n">
         <f aca="false">IFERROR(AVERAGE(I6:I13),"")</f>
@@ -1159,7 +1165,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B17" s="17" t="n">
         <f aca="false">IFERROR(MIN(I6:I13),"")</f>
@@ -1168,7 +1174,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B18" s="17" t="n">
         <f aca="false">IFERROR(MAX(I6:I13),"")</f>
@@ -1177,7 +1183,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B19" s="17" t="n">
         <f aca="false">I5</f>
@@ -1186,19 +1192,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B20" s="17" t="n">
         <f aca="false">IFERROR(250000000/E5,"")</f>
         <v>4023173.47924043</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B21" s="17" t="n">
         <f aca="false">IFERROR(B16*E5,"")</f>

</xml_diff>

<commit_message>
Carmen: T1 piso 8 negociable
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018CaPYB92zD2dguENatYVXw
</commit_message>
<xml_diff>
--- a/finanzas/carmen_competencia_oct2026.xlsx
+++ b/finanzas/carmen_competencia_oct2026.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
   <si>
     <t xml:space="preserve">Competencia — Carmen de Apicalá (conjunto Calle 1 # 11-10) · llamadas 9 oct 2026</t>
   </si>
@@ -168,6 +168,9 @@
   </si>
   <si>
     <t xml:space="preserve">No dice (descripción no lo menciona)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sí (dicho por la asesora)</t>
   </si>
   <si>
     <t xml:space="preserve">Inmobiliaria (Century 21)</t>
@@ -901,13 +904,15 @@
         <v>41</v>
       </c>
       <c r="M6" s="10"/>
-      <c r="N6" s="10"/>
+      <c r="N6" s="10" t="s">
+        <v>42</v>
+      </c>
       <c r="O6" s="10"/>
       <c r="P6" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q6" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="R6" s="12"/>
       <c r="S6" s="10" t="n">
@@ -916,7 +921,7 @@
       <c r="T6" s="12"/>
       <c r="U6" s="10"/>
       <c r="V6" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -924,7 +929,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
@@ -958,7 +963,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
@@ -992,7 +997,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
@@ -1151,12 +1156,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B16" s="17" t="n">
         <f aca="false">IFERROR(AVERAGE(I6:I13),"")</f>
@@ -1165,7 +1170,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B17" s="17" t="n">
         <f aca="false">IFERROR(MIN(I6:I13),"")</f>
@@ -1174,7 +1179,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B18" s="17" t="n">
         <f aca="false">IFERROR(MAX(I6:I13),"")</f>
@@ -1183,7 +1188,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B19" s="17" t="n">
         <f aca="false">I5</f>
@@ -1192,19 +1197,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B20" s="17" t="n">
         <f aca="false">IFERROR(250000000/E5,"")</f>
         <v>4023173.47924043</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B21" s="17" t="n">
         <f aca="false">IFERROR(B16*E5,"")</f>

</xml_diff>

<commit_message>
Carmen: administración $263k y aire acondicionado en T1 piso 8
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018CaPYB92zD2dguENatYVXw
</commit_message>
<xml_diff>
--- a/finanzas/carmen_competencia_oct2026.xlsx
+++ b/finanzas/carmen_competencia_oct2026.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="57">
   <si>
     <t xml:space="preserve">Competencia — Carmen de Apicalá (conjunto Calle 1 # 11-10) · llamadas 9 oct 2026</t>
   </si>
@@ -146,12 +146,15 @@
     <t xml:space="preserve">Dueño (abuelos)</t>
   </si>
   <si>
+    <t xml:space="preserve">~$287k est. (263k × 62,14/57, si se cobra por coeficiente) — confirmar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 (mismo conjunto: Arenitas Riviera PH)</t>
+  </si>
+  <si>
     <t xml:space="preserve">(pendiente)</t>
   </si>
   <si>
-    <t xml:space="preserve">3 (mismo conjunto: Arenitas Riviera PH)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Precio alterno dicho por abuelos: $250M amoblado</t>
   </si>
   <si>
@@ -167,7 +170,7 @@
     <t xml:space="preserve">1 privado cubierto</t>
   </si>
   <si>
-    <t xml:space="preserve">No dice (descripción no lo menciona)</t>
+    <t xml:space="preserve">No amoblado, pero incluye 1 aire acondicionado</t>
   </si>
   <si>
     <t xml:space="preserve">Sí (dicho por la asesora)</t>
@@ -855,13 +858,13 @@
         <v>35</v>
       </c>
       <c r="T5" s="7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U5" s="5" t="s">
         <v>29</v>
       </c>
       <c r="V5" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -869,13 +872,13 @@
         <v>1</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E6" s="11" t="n">
         <v>57</v>
@@ -898,30 +901,32 @@
         <v>-0.00893141945773524</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="M6" s="10"/>
       <c r="N6" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="O6" s="10"/>
       <c r="P6" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Q6" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="R6" s="12"/>
+        <v>45</v>
+      </c>
+      <c r="R6" s="12" t="n">
+        <v>263000</v>
+      </c>
       <c r="S6" s="10" t="n">
         <v>3</v>
       </c>
       <c r="T6" s="12"/>
       <c r="U6" s="10"/>
       <c r="V6" s="10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -929,7 +934,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
@@ -963,7 +968,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
@@ -997,7 +1002,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
@@ -1156,12 +1161,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B16" s="17" t="n">
         <f aca="false">IFERROR(AVERAGE(I6:I13),"")</f>
@@ -1170,7 +1175,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B17" s="17" t="n">
         <f aca="false">IFERROR(MIN(I6:I13),"")</f>
@@ -1179,7 +1184,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B18" s="17" t="n">
         <f aca="false">IFERROR(MAX(I6:I13),"")</f>
@@ -1188,7 +1193,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B19" s="17" t="n">
         <f aca="false">I5</f>
@@ -1197,19 +1202,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B20" s="17" t="n">
         <f aca="false">IFERROR(250000000/E5,"")</f>
         <v>4023173.47924043</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B21" s="17" t="n">
         <f aca="false">IFERROR(B16*E5,"")</f>

</xml_diff>

<commit_message>
Carmen: T1 piso 8 lleva ≥138 días en venta
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018CaPYB92zD2dguENatYVXw
</commit_message>
<xml_diff>
--- a/finanzas/carmen_competencia_oct2026.xlsx
+++ b/finanzas/carmen_competencia_oct2026.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="58">
   <si>
     <t xml:space="preserve">Competencia — Carmen de Apicalá (conjunto Calle 1 # 11-10) · llamadas 9 oct 2026</t>
   </si>
@@ -171,6 +171,9 @@
   </si>
   <si>
     <t xml:space="preserve">No amoblado, pero incluye 1 aire acondicionado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥138 días (última actualización ~24 may 2026, según la página de Century 21)</t>
   </si>
   <si>
     <t xml:space="preserve">Sí (dicho por la asesora)</t>
@@ -906,16 +909,18 @@
       <c r="L6" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="M6" s="10"/>
+      <c r="M6" s="10" t="s">
+        <v>43</v>
+      </c>
       <c r="N6" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="O6" s="10"/>
       <c r="P6" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q6" s="10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="R6" s="12" t="n">
         <v>263000</v>
@@ -926,7 +931,7 @@
       <c r="T6" s="12"/>
       <c r="U6" s="10"/>
       <c r="V6" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -934,7 +939,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
@@ -968,7 +973,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
@@ -1002,7 +1007,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
@@ -1161,12 +1166,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B16" s="17" t="n">
         <f aca="false">IFERROR(AVERAGE(I6:I13),"")</f>
@@ -1175,7 +1180,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B17" s="17" t="n">
         <f aca="false">IFERROR(MIN(I6:I13),"")</f>
@@ -1184,7 +1189,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B18" s="17" t="n">
         <f aca="false">IFERROR(MAX(I6:I13),"")</f>
@@ -1193,7 +1198,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B19" s="17" t="n">
         <f aca="false">I5</f>
@@ -1202,19 +1207,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B20" s="17" t="n">
         <f aca="false">IFERROR(250000000/E5,"")</f>
         <v>4023173.47924043</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B21" s="17" t="n">
         <f aca="false">IFERROR(B16*E5,"")</f>

</xml_diff>

<commit_message>
Carmen: anuncios web del conjunto ($230–250M) y recalibración del rango de precios
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018CaPYB92zD2dguENatYVXw
</commit_message>
<xml_diff>
--- a/finanzas/carmen_competencia_oct2026.xlsx
+++ b/finanzas/carmen_competencia_oct2026.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="71">
   <si>
     <t xml:space="preserve">Competencia — Carmen de Apicalá (conjunto Calle 1 # 11-10) · llamadas 9 oct 2026</t>
   </si>
@@ -192,6 +192,45 @@
   </si>
   <si>
     <t xml:space="preserve">Letrero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metrocuadrado MC6840778 (búsqueda web, sin verificar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 cubierto privado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Construidos 63,3 / privados 55,49 m². Antigüedad 0–5 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metrocuadrado 2469-M6852417 (búsqueda web, sin verificar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conjunto figura como 'La Riviera'. Global Real Estate SAS. Acepta permuta en el norte de Bogotá</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metrocuadrado 23253-M6984946 (búsqueda web, sin verificar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">piso 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 asignados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Piso 6, esquinero. Greenhome SAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mitula / Keeperomega (búsqueda web, sin verificar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">piso 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Piso 5, construido 2022 (admin $150k parece dato dudoso)</t>
   </si>
   <si>
     <t xml:space="preserve">Resumen</t>
@@ -1040,22 +1079,30 @@
       <c r="A10" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="10"/>
+      <c r="B10" s="10" t="s">
+        <v>50</v>
+      </c>
       <c r="C10" s="10"/>
       <c r="D10" s="10"/>
-      <c r="E10" s="11"/>
+      <c r="E10" s="11" t="n">
+        <v>63.3</v>
+      </c>
       <c r="F10" s="10"/>
       <c r="G10" s="10"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="13" t="str">
+      <c r="H10" s="12" t="n">
+        <v>240000000</v>
+      </c>
+      <c r="I10" s="13" t="n">
         <f aca="false">IFERROR(H10/E10,"")</f>
-        <v/>
-      </c>
-      <c r="J10" s="14" t="str">
+        <v>3791469.1943128</v>
+      </c>
+      <c r="J10" s="14" t="n">
         <f aca="false">IFERROR(I10/$I$5-1,"")</f>
-        <v/>
-      </c>
-      <c r="K10" s="10"/>
+        <v>0.0709177078845327</v>
+      </c>
+      <c r="K10" s="10" t="s">
+        <v>51</v>
+      </c>
       <c r="L10" s="10"/>
       <c r="M10" s="10"/>
       <c r="N10" s="10"/>
@@ -1066,26 +1113,34 @@
       <c r="S10" s="10"/>
       <c r="T10" s="12"/>
       <c r="U10" s="10"/>
-      <c r="V10" s="10"/>
+      <c r="V10" s="10" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="10"/>
+      <c r="B11" s="10" t="s">
+        <v>53</v>
+      </c>
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
-      <c r="E11" s="11"/>
+      <c r="E11" s="11" t="n">
+        <v>63</v>
+      </c>
       <c r="F11" s="10"/>
       <c r="G11" s="10"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="13" t="str">
+      <c r="H11" s="12" t="n">
+        <v>240000000</v>
+      </c>
+      <c r="I11" s="13" t="n">
         <f aca="false">IFERROR(H11/E11,"")</f>
-        <v/>
-      </c>
-      <c r="J11" s="14" t="str">
+        <v>3809523.80952381</v>
+      </c>
+      <c r="J11" s="14" t="n">
         <f aca="false">IFERROR(I11/$I$5-1,"")</f>
-        <v/>
+        <v>0.0760173160173161</v>
       </c>
       <c r="K11" s="10"/>
       <c r="L11" s="10"/>
@@ -1094,93 +1149,125 @@
       <c r="O11" s="10"/>
       <c r="P11" s="10"/>
       <c r="Q11" s="10"/>
-      <c r="R11" s="12"/>
+      <c r="R11" s="12" t="n">
+        <v>300000</v>
+      </c>
       <c r="S11" s="10"/>
       <c r="T11" s="12"/>
       <c r="U11" s="10"/>
-      <c r="V11" s="10"/>
+      <c r="V11" s="10" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="10"/>
+      <c r="B12" s="10" t="s">
+        <v>55</v>
+      </c>
       <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="11"/>
+      <c r="D12" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>63</v>
+      </c>
       <c r="F12" s="10"/>
       <c r="G12" s="10"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="13" t="str">
+      <c r="H12" s="12" t="n">
+        <v>250000000</v>
+      </c>
+      <c r="I12" s="13" t="n">
         <f aca="false">IFERROR(H12/E12,"")</f>
-        <v/>
-      </c>
-      <c r="J12" s="14" t="str">
+        <v>3968253.96825397</v>
+      </c>
+      <c r="J12" s="14" t="n">
         <f aca="false">IFERROR(I12/$I$5-1,"")</f>
-        <v/>
-      </c>
-      <c r="K12" s="10"/>
+        <v>0.120851370851371</v>
+      </c>
+      <c r="K12" s="10" t="s">
+        <v>57</v>
+      </c>
       <c r="L12" s="10"/>
       <c r="M12" s="10"/>
       <c r="N12" s="10"/>
       <c r="O12" s="10"/>
       <c r="P12" s="10"/>
       <c r="Q12" s="10"/>
-      <c r="R12" s="12"/>
+      <c r="R12" s="12" t="n">
+        <v>308000</v>
+      </c>
       <c r="S12" s="10"/>
       <c r="T12" s="12"/>
       <c r="U12" s="10"/>
-      <c r="V12" s="10"/>
+      <c r="V12" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="10"/>
+      <c r="B13" s="10" t="s">
+        <v>59</v>
+      </c>
       <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="11"/>
+      <c r="D13" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>63</v>
+      </c>
       <c r="F13" s="10"/>
       <c r="G13" s="10"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="13" t="str">
+      <c r="H13" s="12" t="n">
+        <v>230000000</v>
+      </c>
+      <c r="I13" s="13" t="n">
         <f aca="false">IFERROR(H13/E13,"")</f>
-        <v/>
-      </c>
-      <c r="J13" s="14" t="str">
+        <v>3650793.65079365</v>
+      </c>
+      <c r="J13" s="14" t="n">
         <f aca="false">IFERROR(I13/$I$5-1,"")</f>
-        <v/>
-      </c>
-      <c r="K13" s="10"/>
+        <v>0.0311832611832612</v>
+      </c>
+      <c r="K13" s="10" t="s">
+        <v>61</v>
+      </c>
       <c r="L13" s="10"/>
       <c r="M13" s="10"/>
       <c r="N13" s="10"/>
       <c r="O13" s="10"/>
       <c r="P13" s="10"/>
       <c r="Q13" s="10"/>
-      <c r="R13" s="12"/>
+      <c r="R13" s="12" t="n">
+        <v>150000</v>
+      </c>
       <c r="S13" s="10"/>
       <c r="T13" s="12"/>
       <c r="U13" s="10"/>
-      <c r="V13" s="10"/>
+      <c r="V13" s="10" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="B16" s="17" t="n">
         <f aca="false">IFERROR(AVERAGE(I6:I13),"")</f>
-        <v>3508771.92982456</v>
+        <v>3745762.51054176</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="B17" s="17" t="n">
         <f aca="false">IFERROR(MIN(I6:I13),"")</f>
@@ -1189,16 +1276,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="B18" s="17" t="n">
         <f aca="false">IFERROR(MAX(I6:I13),"")</f>
-        <v>3508771.92982456</v>
+        <v>3968253.96825397</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="B19" s="17" t="n">
         <f aca="false">I5</f>
@@ -1207,23 +1294,23 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="B20" s="17" t="n">
         <f aca="false">IFERROR(250000000/E5,"")</f>
         <v>4023173.47924043</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="B21" s="17" t="n">
         <f aca="false">IFERROR(B16*E5,"")</f>
-        <v>218035087.719298</v>
+        <v>232761682.405065</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Carmen: $250M retirado, $240M re-publicado a $220M
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018CaPYB92zD2dguENatYVXw
</commit_message>
<xml_diff>
--- a/finanzas/carmen_competencia_oct2026.xlsx
+++ b/finanzas/carmen_competencia_oct2026.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="72">
   <si>
     <t xml:space="preserve">Competencia — Carmen de Apicalá (conjunto Calle 1 # 11-10) · llamadas 9 oct 2026</t>
   </si>
@@ -194,13 +194,16 @@
     <t xml:space="preserve">Letrero</t>
   </si>
   <si>
-    <t xml:space="preserve">Metrocuadrado MC6840778 (búsqueda web, sin verificar)</t>
+    <t xml:space="preserve">Metrocuadrado MC6840778 (re-publicado a $220M)</t>
   </si>
   <si>
     <t xml:space="preserve">1 cubierto privado</t>
   </si>
   <si>
-    <t xml:space="preserve">Construidos 63,3 / privados 55,49 m². Antigüedad 0–5 años</t>
+    <t xml:space="preserve">Ya rebajó $20M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bajó de $240M a $220M: nueva publicación más reciente del mismo apto (confirmado por Felipe 9 oct). Construidos 63,3 / privados 55,49 m²</t>
   </si>
   <si>
     <t xml:space="preserve">Metrocuadrado 2469-M6852417 (búsqueda web, sin verificar)</t>
@@ -209,7 +212,7 @@
     <t xml:space="preserve">Conjunto figura como 'La Riviera'. Global Real Estate SAS. Acepta permuta en el norte de Bogotá</t>
   </si>
   <si>
-    <t xml:space="preserve">Metrocuadrado 23253-M6984946 (búsqueda web, sin verificar)</t>
+    <t xml:space="preserve">Metrocuadrado 23253-M6984946 — YA NO ESTÁ PUBLICADO</t>
   </si>
   <si>
     <t xml:space="preserve">piso 6</t>
@@ -218,7 +221,7 @@
     <t xml:space="preserve">2 asignados</t>
   </si>
   <si>
-    <t xml:space="preserve">Piso 6, esquinero. Greenhome SAS</t>
+    <t xml:space="preserve">Pedía $250M (piso 6, esquinero, 2 parqueaderos, admin $308k). Retirado: ¿vendido o desistió? Desconocido</t>
   </si>
   <si>
     <t xml:space="preserve">Mitula / Keeperomega (búsqueda web, sin verificar)</t>
@@ -1090,22 +1093,24 @@
       <c r="F10" s="10"/>
       <c r="G10" s="10"/>
       <c r="H10" s="12" t="n">
-        <v>240000000</v>
+        <v>220000000</v>
       </c>
       <c r="I10" s="13" t="n">
         <f aca="false">IFERROR(H10/E10,"")</f>
-        <v>3791469.1943128</v>
+        <v>3475513.42812006</v>
       </c>
       <c r="J10" s="14" t="n">
         <f aca="false">IFERROR(I10/$I$5-1,"")</f>
-        <v>0.0709177078845327</v>
+        <v>-0.0183254344391784</v>
       </c>
       <c r="K10" s="10" t="s">
         <v>51</v>
       </c>
       <c r="L10" s="10"/>
       <c r="M10" s="10"/>
-      <c r="N10" s="10"/>
+      <c r="N10" s="10" t="s">
+        <v>52</v>
+      </c>
       <c r="O10" s="10"/>
       <c r="P10" s="10"/>
       <c r="Q10" s="10"/>
@@ -1114,7 +1119,7 @@
       <c r="T10" s="12"/>
       <c r="U10" s="10"/>
       <c r="V10" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1122,7 +1127,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
@@ -1156,7 +1161,7 @@
       <c r="T11" s="12"/>
       <c r="U11" s="10"/>
       <c r="V11" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1164,11 +1169,11 @@
         <v>7</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C12" s="10"/>
       <c r="D12" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>63</v>
@@ -1187,7 +1192,7 @@
         <v>0.120851370851371</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="L12" s="10"/>
       <c r="M12" s="10"/>
@@ -1202,7 +1207,7 @@
       <c r="T12" s="12"/>
       <c r="U12" s="10"/>
       <c r="V12" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1210,11 +1215,11 @@
         <v>8</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E13" s="11" t="n">
         <v>63</v>
@@ -1233,7 +1238,7 @@
         <v>0.0311832611832612</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="L13" s="10"/>
       <c r="M13" s="10"/>
@@ -1248,35 +1253,35 @@
       <c r="T13" s="12"/>
       <c r="U13" s="10"/>
       <c r="V13" s="10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B16" s="17" t="n">
         <f aca="false">IFERROR(AVERAGE(I6:I13),"")</f>
-        <v>3745762.51054176</v>
+        <v>3682571.35730321</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B17" s="17" t="n">
         <f aca="false">IFERROR(MIN(I6:I13),"")</f>
-        <v>3508771.92982456</v>
+        <v>3475513.42812006</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B18" s="17" t="n">
         <f aca="false">IFERROR(MAX(I6:I13),"")</f>
@@ -1285,7 +1290,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B19" s="17" t="n">
         <f aca="false">I5</f>
@@ -1294,23 +1299,23 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B20" s="17" t="n">
         <f aca="false">IFERROR(250000000/E5,"")</f>
         <v>4023173.47924043</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B21" s="17" t="n">
         <f aca="false">IFERROR(B16*E5,"")</f>
-        <v>232761682.405065</v>
+        <v>228834984.142822</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Carmen: administración $275k, predial ~$60k/año (sin desenglobe), BBQ
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018CaPYB92zD2dguENatYVXw
</commit_message>
<xml_diff>
--- a/finanzas/carmen_competencia_oct2026.xlsx
+++ b/finanzas/carmen_competencia_oct2026.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="70">
   <si>
     <t xml:space="preserve">Competencia — Carmen de Apicalá (conjunto Calle 1 # 11-10) · llamadas 9 oct 2026</t>
   </si>
@@ -146,16 +146,10 @@
     <t xml:space="preserve">Dueño (abuelos)</t>
   </si>
   <si>
-    <t xml:space="preserve">~$287k est. (263k × 62,14/57, si se cobra por coeficiente) — confirmar</t>
-  </si>
-  <si>
     <t xml:space="preserve">3 (mismo conjunto: Arenitas Riviera PH)</t>
   </si>
   <si>
-    <t xml:space="preserve">(pendiente)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Precio alterno dicho por abuelos: $250M amoblado</t>
+    <t xml:space="preserve">Precio único $220M (decidido con el abuelo, viaje 8–10 oct). Predial ~$60k/año: conjunto sin desenglobar</t>
   </si>
   <si>
     <t xml:space="preserve">Letrero · Century 21 (ficha ID 149314)</t>
@@ -896,20 +890,20 @@
       <c r="Q5" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="R5" s="7" t="s">
+      <c r="R5" s="7" t="n">
+        <v>275000</v>
+      </c>
+      <c r="S5" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="S5" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="T5" s="7" t="s">
-        <v>36</v>
+      <c r="T5" s="7" t="n">
+        <v>60000</v>
       </c>
       <c r="U5" s="5" t="s">
         <v>29</v>
       </c>
       <c r="V5" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -917,13 +911,13 @@
         <v>1</v>
       </c>
       <c r="B6" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>38</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>40</v>
       </c>
       <c r="E6" s="11" t="n">
         <v>57</v>
@@ -946,23 +940,23 @@
         <v>-0.00893141945773524</v>
       </c>
       <c r="K6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="L6" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="M6" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="L6" s="10" t="s">
+      <c r="N6" s="10" t="s">
         <v>42</v>
-      </c>
-      <c r="M6" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="N6" s="10" t="s">
-        <v>44</v>
       </c>
       <c r="O6" s="10"/>
       <c r="P6" s="10" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="Q6" s="10" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="R6" s="12" t="n">
         <v>263000</v>
@@ -973,7 +967,7 @@
       <c r="T6" s="12"/>
       <c r="U6" s="10"/>
       <c r="V6" s="10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -981,7 +975,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
@@ -1015,7 +1009,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
@@ -1049,7 +1043,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
@@ -1083,7 +1077,7 @@
         <v>5</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="10"/>
@@ -1104,12 +1098,12 @@
         <v>-0.0183254344391784</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L10" s="10"/>
       <c r="M10" s="10"/>
       <c r="N10" s="10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="O10" s="10"/>
       <c r="P10" s="10"/>
@@ -1119,7 +1113,7 @@
       <c r="T10" s="12"/>
       <c r="U10" s="10"/>
       <c r="V10" s="10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1127,7 +1121,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
@@ -1161,7 +1155,7 @@
       <c r="T11" s="12"/>
       <c r="U11" s="10"/>
       <c r="V11" s="10" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1169,11 +1163,11 @@
         <v>7</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C12" s="10"/>
       <c r="D12" s="10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>63</v>
@@ -1192,7 +1186,7 @@
         <v>0.120851370851371</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L12" s="10"/>
       <c r="M12" s="10"/>
@@ -1207,7 +1201,7 @@
       <c r="T12" s="12"/>
       <c r="U12" s="10"/>
       <c r="V12" s="10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1215,11 +1209,11 @@
         <v>8</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="10" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E13" s="11" t="n">
         <v>63</v>
@@ -1238,7 +1232,7 @@
         <v>0.0311832611832612</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="L13" s="10"/>
       <c r="M13" s="10"/>
@@ -1253,17 +1247,17 @@
       <c r="T13" s="12"/>
       <c r="U13" s="10"/>
       <c r="V13" s="10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B16" s="17" t="n">
         <f aca="false">IFERROR(AVERAGE(I6:I13),"")</f>
@@ -1272,7 +1266,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B17" s="17" t="n">
         <f aca="false">IFERROR(MIN(I6:I13),"")</f>
@@ -1281,7 +1275,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B18" s="17" t="n">
         <f aca="false">IFERROR(MAX(I6:I13),"")</f>
@@ -1290,7 +1284,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B19" s="17" t="n">
         <f aca="false">I5</f>
@@ -1299,19 +1293,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B20" s="17" t="n">
         <f aca="false">IFERROR(250000000/E5,"")</f>
         <v>4023173.47924043</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B21" s="17" t="n">
         <f aca="false">IFERROR(B16*E5,"")</f>

</xml_diff>